<commit_message>
Rediseño: cuadro en espejo, línea de tiempo de horarios y panel con PIN sobre Supabase
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FKDmR3ZQYFSst4xhjJhdPn
</commit_message>
<xml_diff>
--- a/datos/fixture.xlsx
+++ b/datos/fixture.xlsx
@@ -139,24 +139,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -175,9 +165,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
@@ -499,7 +487,7 @@
         </is>
       </c>
       <c r="E1" s="4" t="n"/>
-      <c r="F1" s="5" t="n"/>
+      <c r="F1" s="21" t="n"/>
       <c r="G1" s="6" t="n"/>
       <c r="H1" s="7" t="inlineStr">
         <is>
@@ -512,7 +500,7 @@
           <t>RONDA DE 64</t>
         </is>
       </c>
-      <c r="K1" s="5" t="n"/>
+      <c r="K1" s="21" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="10" t="n">
@@ -554,7 +542,7 @@
           <t>VS</t>
         </is>
       </c>
-      <c r="J2" s="15" t="n"/>
+      <c r="J2" s="19" t="n"/>
       <c r="K2" s="10" t="n">
         <v>64</v>
       </c>
@@ -642,7 +630,7 @@
           <t>VS</t>
         </is>
       </c>
-      <c r="J4" s="15" t="n"/>
+      <c r="J4" s="19" t="n"/>
       <c r="K4" s="10" t="n">
         <v>62</v>
       </c>
@@ -685,7 +673,7 @@
           <t>VS</t>
         </is>
       </c>
-      <c r="J5" s="15" t="n"/>
+      <c r="J5" s="19" t="n"/>
       <c r="K5" s="10" t="n">
         <v>61</v>
       </c>
@@ -730,7 +718,7 @@
           <t>VS</t>
         </is>
       </c>
-      <c r="J6" s="15" t="n"/>
+      <c r="J6" s="19" t="n"/>
       <c r="K6" s="10" t="n">
         <v>60</v>
       </c>
@@ -857,11 +845,7 @@
       <c r="G9" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>NESTOR MARIN 19</t>
-        </is>
-      </c>
+      <c r="H9" s="11" t="n"/>
       <c r="I9" s="12" t="inlineStr">
         <is>
           <t>VS</t>
@@ -2035,11 +2019,11 @@
       <c r="F34" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G34" s="5" t="n"/>
+      <c r="G34" s="21" t="n"/>
       <c r="H34" s="21" t="n"/>
-      <c r="I34" s="5" t="n"/>
+      <c r="I34" s="21" t="n"/>
       <c r="J34" s="21" t="n"/>
-      <c r="K34" s="5" t="n"/>
+      <c r="K34" s="21" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="16" t="n">
@@ -2066,11 +2050,11 @@
       <c r="F35" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G35" s="5" t="n"/>
+      <c r="G35" s="21" t="n"/>
       <c r="H35" s="21" t="n"/>
-      <c r="I35" s="5" t="n"/>
+      <c r="I35" s="21" t="n"/>
       <c r="J35" s="21" t="n"/>
-      <c r="K35" s="5" t="n"/>
+      <c r="K35" s="21" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="16" t="n">
@@ -2099,11 +2083,11 @@
           <t>11A</t>
         </is>
       </c>
-      <c r="G36" s="5" t="n"/>
+      <c r="G36" s="21" t="n"/>
       <c r="H36" s="21" t="n"/>
-      <c r="I36" s="5" t="n"/>
-      <c r="J36" s="5" t="n"/>
-      <c r="K36" s="5" t="n"/>
+      <c r="I36" s="21" t="n"/>
+      <c r="J36" s="21" t="n"/>
+      <c r="K36" s="21" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="16" t="n">
@@ -2130,11 +2114,11 @@
       <c r="F37" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G37" s="5" t="n"/>
+      <c r="G37" s="21" t="n"/>
       <c r="H37" s="21" t="n"/>
-      <c r="I37" s="5" t="n"/>
+      <c r="I37" s="21" t="n"/>
       <c r="J37" s="22" t="n"/>
-      <c r="K37" s="5" t="n"/>
+      <c r="K37" s="21" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="16" t="n">
@@ -2163,11 +2147,11 @@
           <t>11A</t>
         </is>
       </c>
-      <c r="G38" s="5" t="n"/>
+      <c r="G38" s="21" t="n"/>
       <c r="H38" s="21" t="n"/>
-      <c r="I38" s="5" t="n"/>
-      <c r="J38" s="5" t="n"/>
-      <c r="K38" s="5" t="n"/>
+      <c r="I38" s="21" t="n"/>
+      <c r="J38" s="21" t="n"/>
+      <c r="K38" s="21" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="16" t="n">
@@ -2196,11 +2180,11 @@
           <t>11A</t>
         </is>
       </c>
-      <c r="G39" s="5" t="n"/>
+      <c r="G39" s="21" t="n"/>
       <c r="H39" s="21" t="n"/>
-      <c r="I39" s="5" t="n"/>
+      <c r="I39" s="21" t="n"/>
       <c r="J39" s="21" t="n"/>
-      <c r="K39" s="5" t="n"/>
+      <c r="K39" s="21" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="16" t="n">
@@ -2229,11 +2213,11 @@
           <t>11A</t>
         </is>
       </c>
-      <c r="G40" s="5" t="n"/>
+      <c r="G40" s="21" t="n"/>
       <c r="H40" s="21" t="n"/>
-      <c r="I40" s="5" t="n"/>
+      <c r="I40" s="21" t="n"/>
       <c r="J40" s="21" t="n"/>
-      <c r="K40" s="5" t="n"/>
+      <c r="K40" s="21" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="16" t="n">
@@ -2260,11 +2244,11 @@
       <c r="F41" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G41" s="5" t="n"/>
+      <c r="G41" s="21" t="n"/>
       <c r="H41" s="21" t="n"/>
-      <c r="I41" s="5" t="n"/>
+      <c r="I41" s="21" t="n"/>
       <c r="J41" s="21" t="n"/>
-      <c r="K41" s="5" t="n"/>
+      <c r="K41" s="21" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="16" t="n">
@@ -2291,11 +2275,11 @@
       <c r="F42" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="5" t="n"/>
-      <c r="I42" s="5" t="n"/>
-      <c r="J42" s="5" t="n"/>
-      <c r="K42" s="5" t="n"/>
+      <c r="G42" s="21" t="n"/>
+      <c r="H42" s="21" t="n"/>
+      <c r="I42" s="21" t="n"/>
+      <c r="J42" s="21" t="n"/>
+      <c r="K42" s="21" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="16" t="n">
@@ -2322,11 +2306,11 @@
       <c r="F43" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G43" s="5" t="n"/>
-      <c r="H43" s="5" t="n"/>
-      <c r="I43" s="5" t="n"/>
-      <c r="J43" s="5" t="n"/>
-      <c r="K43" s="5" t="n"/>
+      <c r="G43" s="21" t="n"/>
+      <c r="H43" s="21" t="n"/>
+      <c r="I43" s="21" t="n"/>
+      <c r="J43" s="21" t="n"/>
+      <c r="K43" s="21" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="16" t="n">
@@ -2355,11 +2339,11 @@
           <t>11A</t>
         </is>
       </c>
-      <c r="G44" s="5" t="n"/>
-      <c r="H44" s="5" t="n"/>
-      <c r="I44" s="5" t="n"/>
-      <c r="J44" s="5" t="n"/>
-      <c r="K44" s="5" t="n"/>
+      <c r="G44" s="21" t="n"/>
+      <c r="H44" s="21" t="n"/>
+      <c r="I44" s="21" t="n"/>
+      <c r="J44" s="21" t="n"/>
+      <c r="K44" s="21" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="16" t="n">
@@ -2388,11 +2372,11 @@
           <t>11A</t>
         </is>
       </c>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="5" t="n"/>
-      <c r="I45" s="5" t="n"/>
-      <c r="J45" s="5" t="n"/>
-      <c r="K45" s="5" t="n"/>
+      <c r="G45" s="21" t="n"/>
+      <c r="H45" s="21" t="n"/>
+      <c r="I45" s="21" t="n"/>
+      <c r="J45" s="21" t="n"/>
+      <c r="K45" s="21" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="16" t="n">
@@ -2421,11 +2405,11 @@
           <t>11A</t>
         </is>
       </c>
-      <c r="G46" s="5" t="n"/>
-      <c r="H46" s="5" t="n"/>
-      <c r="I46" s="5" t="n"/>
-      <c r="J46" s="5" t="n"/>
-      <c r="K46" s="5" t="n"/>
+      <c r="G46" s="21" t="n"/>
+      <c r="H46" s="21" t="n"/>
+      <c r="I46" s="21" t="n"/>
+      <c r="J46" s="21" t="n"/>
+      <c r="K46" s="21" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="16" t="n">
@@ -2454,11 +2438,11 @@
           <t>11A</t>
         </is>
       </c>
-      <c r="G47" s="5" t="n"/>
-      <c r="H47" s="5" t="n"/>
-      <c r="I47" s="5" t="n"/>
-      <c r="J47" s="5" t="n"/>
-      <c r="K47" s="5" t="n"/>
+      <c r="G47" s="21" t="n"/>
+      <c r="H47" s="21" t="n"/>
+      <c r="I47" s="21" t="n"/>
+      <c r="J47" s="21" t="n"/>
+      <c r="K47" s="21" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n">
@@ -2487,11 +2471,11 @@
           <t>12A</t>
         </is>
       </c>
-      <c r="G48" s="5" t="n"/>
-      <c r="H48" s="5" t="n"/>
-      <c r="I48" s="5" t="n"/>
-      <c r="J48" s="5" t="n"/>
-      <c r="K48" s="5" t="n"/>
+      <c r="G48" s="21" t="n"/>
+      <c r="H48" s="21" t="n"/>
+      <c r="I48" s="21" t="n"/>
+      <c r="J48" s="21" t="n"/>
+      <c r="K48" s="21" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="16" t="n">
@@ -2518,11 +2502,11 @@
       <c r="F49" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G49" s="5" t="n"/>
-      <c r="H49" s="5" t="n"/>
-      <c r="I49" s="5" t="n"/>
-      <c r="J49" s="5" t="n"/>
-      <c r="K49" s="5" t="n"/>
+      <c r="G49" s="21" t="n"/>
+      <c r="H49" s="21" t="n"/>
+      <c r="I49" s="21" t="n"/>
+      <c r="J49" s="21" t="n"/>
+      <c r="K49" s="21" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="16" t="n">
@@ -2549,11 +2533,11 @@
       <c r="F50" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="5" t="n"/>
-      <c r="I50" s="5" t="n"/>
-      <c r="J50" s="5" t="n"/>
-      <c r="K50" s="5" t="n"/>
+      <c r="G50" s="21" t="n"/>
+      <c r="H50" s="21" t="n"/>
+      <c r="I50" s="21" t="n"/>
+      <c r="J50" s="21" t="n"/>
+      <c r="K50" s="21" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="16" t="n">
@@ -2582,11 +2566,11 @@
           <t>12A</t>
         </is>
       </c>
-      <c r="G51" s="5" t="n"/>
-      <c r="H51" s="5" t="n"/>
-      <c r="I51" s="5" t="n"/>
-      <c r="J51" s="5" t="n"/>
-      <c r="K51" s="5" t="n"/>
+      <c r="G51" s="21" t="n"/>
+      <c r="H51" s="21" t="n"/>
+      <c r="I51" s="21" t="n"/>
+      <c r="J51" s="21" t="n"/>
+      <c r="K51" s="21" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="16" t="n">
@@ -2613,11 +2597,11 @@
       <c r="F52" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G52" s="5" t="n"/>
-      <c r="H52" s="5" t="n"/>
-      <c r="I52" s="5" t="n"/>
-      <c r="J52" s="5" t="n"/>
-      <c r="K52" s="5" t="n"/>
+      <c r="G52" s="21" t="n"/>
+      <c r="H52" s="21" t="n"/>
+      <c r="I52" s="21" t="n"/>
+      <c r="J52" s="21" t="n"/>
+      <c r="K52" s="21" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="16" t="n">
@@ -2644,11 +2628,11 @@
       <c r="F53" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G53" s="5" t="n"/>
-      <c r="H53" s="5" t="n"/>
-      <c r="I53" s="5" t="n"/>
-      <c r="J53" s="5" t="n"/>
-      <c r="K53" s="5" t="n"/>
+      <c r="G53" s="21" t="n"/>
+      <c r="H53" s="21" t="n"/>
+      <c r="I53" s="21" t="n"/>
+      <c r="J53" s="21" t="n"/>
+      <c r="K53" s="21" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="16" t="n">
@@ -2675,11 +2659,11 @@
       <c r="F54" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G54" s="5" t="n"/>
-      <c r="H54" s="5" t="n"/>
-      <c r="I54" s="5" t="n"/>
-      <c r="J54" s="5" t="n"/>
-      <c r="K54" s="5" t="n"/>
+      <c r="G54" s="21" t="n"/>
+      <c r="H54" s="21" t="n"/>
+      <c r="I54" s="21" t="n"/>
+      <c r="J54" s="21" t="n"/>
+      <c r="K54" s="21" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="16" t="n">
@@ -2708,11 +2692,11 @@
           <t>12A</t>
         </is>
       </c>
-      <c r="G55" s="5" t="n"/>
-      <c r="H55" s="5" t="n"/>
-      <c r="I55" s="5" t="n"/>
-      <c r="J55" s="5" t="n"/>
-      <c r="K55" s="5" t="n"/>
+      <c r="G55" s="21" t="n"/>
+      <c r="H55" s="21" t="n"/>
+      <c r="I55" s="21" t="n"/>
+      <c r="J55" s="21" t="n"/>
+      <c r="K55" s="21" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="n">
@@ -2739,11 +2723,11 @@
       <c r="F56" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G56" s="5" t="n"/>
-      <c r="H56" s="5" t="n"/>
-      <c r="I56" s="5" t="n"/>
-      <c r="J56" s="5" t="n"/>
-      <c r="K56" s="5" t="n"/>
+      <c r="G56" s="21" t="n"/>
+      <c r="H56" s="21" t="n"/>
+      <c r="I56" s="21" t="n"/>
+      <c r="J56" s="21" t="n"/>
+      <c r="K56" s="21" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="16" t="n">
@@ -2772,11 +2756,11 @@
           <t>12A</t>
         </is>
       </c>
-      <c r="G57" s="5" t="n"/>
-      <c r="H57" s="5" t="n"/>
-      <c r="I57" s="5" t="n"/>
-      <c r="J57" s="5" t="n"/>
-      <c r="K57" s="5" t="n"/>
+      <c r="G57" s="21" t="n"/>
+      <c r="H57" s="21" t="n"/>
+      <c r="I57" s="21" t="n"/>
+      <c r="J57" s="21" t="n"/>
+      <c r="K57" s="21" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="16" t="n">
@@ -2805,11 +2789,11 @@
           <t>12A</t>
         </is>
       </c>
-      <c r="G58" s="5" t="n"/>
-      <c r="H58" s="5" t="n"/>
-      <c r="I58" s="5" t="n"/>
-      <c r="J58" s="5" t="n"/>
-      <c r="K58" s="5" t="n"/>
+      <c r="G58" s="21" t="n"/>
+      <c r="H58" s="21" t="n"/>
+      <c r="I58" s="21" t="n"/>
+      <c r="J58" s="21" t="n"/>
+      <c r="K58" s="21" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="16" t="n">
@@ -2833,12 +2817,12 @@
       <c r="E59" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="F59" s="5" t="n"/>
-      <c r="G59" s="5" t="n"/>
-      <c r="H59" s="5" t="n"/>
-      <c r="I59" s="5" t="n"/>
-      <c r="J59" s="5" t="n"/>
-      <c r="K59" s="5" t="n"/>
+      <c r="F59" s="21" t="n"/>
+      <c r="G59" s="21" t="n"/>
+      <c r="H59" s="21" t="n"/>
+      <c r="I59" s="21" t="n"/>
+      <c r="J59" s="21" t="n"/>
+      <c r="K59" s="21" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="16" t="n">
@@ -2867,11 +2851,11 @@
           <t>12A</t>
         </is>
       </c>
-      <c r="G60" s="5" t="n"/>
-      <c r="H60" s="5" t="n"/>
-      <c r="I60" s="5" t="n"/>
-      <c r="J60" s="5" t="n"/>
-      <c r="K60" s="5" t="n"/>
+      <c r="G60" s="21" t="n"/>
+      <c r="H60" s="21" t="n"/>
+      <c r="I60" s="21" t="n"/>
+      <c r="J60" s="21" t="n"/>
+      <c r="K60" s="21" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="16" t="n">
@@ -2900,11 +2884,11 @@
           <t>12A</t>
         </is>
       </c>
-      <c r="G61" s="5" t="n"/>
-      <c r="H61" s="5" t="n"/>
-      <c r="I61" s="5" t="n"/>
-      <c r="J61" s="5" t="n"/>
-      <c r="K61" s="5" t="n"/>
+      <c r="G61" s="21" t="n"/>
+      <c r="H61" s="21" t="n"/>
+      <c r="I61" s="21" t="n"/>
+      <c r="J61" s="21" t="n"/>
+      <c r="K61" s="21" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="16" t="n">
@@ -2933,11 +2917,11 @@
           <t>12A</t>
         </is>
       </c>
-      <c r="G62" s="5" t="n"/>
-      <c r="H62" s="5" t="n"/>
-      <c r="I62" s="5" t="n"/>
-      <c r="J62" s="5" t="n"/>
-      <c r="K62" s="5" t="n"/>
+      <c r="G62" s="21" t="n"/>
+      <c r="H62" s="21" t="n"/>
+      <c r="I62" s="21" t="n"/>
+      <c r="J62" s="21" t="n"/>
+      <c r="K62" s="21" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="16" t="n">
@@ -2966,11 +2950,11 @@
           <t>12A</t>
         </is>
       </c>
-      <c r="G63" s="5" t="n"/>
-      <c r="H63" s="5" t="n"/>
-      <c r="I63" s="5" t="n"/>
-      <c r="J63" s="5" t="n"/>
-      <c r="K63" s="5" t="n"/>
+      <c r="G63" s="21" t="n"/>
+      <c r="H63" s="21" t="n"/>
+      <c r="I63" s="21" t="n"/>
+      <c r="J63" s="21" t="n"/>
+      <c r="K63" s="21" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="16" t="n">
@@ -2999,35 +2983,35 @@
           <t>12A</t>
         </is>
       </c>
-      <c r="G64" s="5" t="n"/>
-      <c r="H64" s="5" t="n"/>
-      <c r="I64" s="5" t="n"/>
-      <c r="J64" s="5" t="n"/>
-      <c r="K64" s="5" t="n"/>
+      <c r="G64" s="21" t="n"/>
+      <c r="H64" s="21" t="n"/>
+      <c r="I64" s="21" t="n"/>
+      <c r="J64" s="21" t="n"/>
+      <c r="K64" s="21" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" t="n">
+      <c r="A65" s="0" t="n">
         <v>64</v>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="0" t="inlineStr">
         <is>
           <t>SEBASTIAN DIAZ</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>VS</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
+      <c r="C65" s="0" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="D65" s="0" t="inlineStr">
         <is>
           <t>MIGUEL POVEDA</t>
         </is>
       </c>
-      <c r="E65" t="n">
+      <c r="E65" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="0" t="inlineStr">
         <is>
           <t>12A</t>
         </is>

</xml_diff>